<commit_message>
updating to match new data
</commit_message>
<xml_diff>
--- a/data/correlated/Pros_96 plot_Seq_Yeld_25.xlsx
+++ b/data/correlated/Pros_96 plot_Seq_Yeld_25.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ndusbpos-my.sharepoint.com/personal/md_m_rahman_ndus_edu/Documents/Microsoft Copilot Chat Files/Desktop/UCLA_Genomic_Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhenyusong/Desktop/mae199/flax-and-canola/data/correlated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{95D745FF-B8E3-40AB-AD1A-2DCF3E42FAFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F5D8B45-D663-4F70-A6A0-DA2C1C557192}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03ADE867-9305-3847-A939-781476737956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9345" yWindow="90" windowWidth="19695" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9340" yWindow="880" windowWidth="19700" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pheno" sheetId="3" r:id="rId1"/>
@@ -28,9 +28,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -701,13 +698,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECA49917-DA91-4F61-B011-B8E7083118F2}">
   <dimension ref="A1:D97"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="12.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="12.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -721,7 +718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1128</v>
       </c>
@@ -735,7 +732,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1129</v>
       </c>
@@ -749,7 +746,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>1130</v>
       </c>
@@ -763,7 +760,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>1002</v>
       </c>
@@ -777,7 +774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>1005</v>
       </c>
@@ -791,7 +788,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>1006</v>
       </c>
@@ -805,7 +802,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>1007</v>
       </c>
@@ -819,7 +816,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>1008</v>
       </c>
@@ -833,7 +830,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>1009</v>
       </c>
@@ -847,7 +844,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>1012</v>
       </c>
@@ -861,7 +858,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>1015</v>
       </c>
@@ -875,7 +872,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>1016</v>
       </c>
@@ -889,7 +886,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>1131</v>
       </c>
@@ -903,7 +900,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>1018</v>
       </c>
@@ -917,7 +914,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>1019</v>
       </c>
@@ -931,7 +928,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>1132</v>
       </c>
@@ -945,7 +942,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>1024</v>
       </c>
@@ -959,7 +956,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>1025</v>
       </c>
@@ -973,7 +970,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>1133</v>
       </c>
@@ -987,7 +984,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>1028</v>
       </c>
@@ -1001,7 +998,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>1135</v>
       </c>
@@ -1015,7 +1012,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>1030</v>
       </c>
@@ -1029,7 +1026,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>1031</v>
       </c>
@@ -1043,7 +1040,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>1032</v>
       </c>
@@ -1057,7 +1054,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>1034</v>
       </c>
@@ -1071,7 +1068,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>1136</v>
       </c>
@@ -1085,7 +1082,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>1037</v>
       </c>
@@ -1099,7 +1096,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>1138</v>
       </c>
@@ -1113,7 +1110,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>1044</v>
       </c>
@@ -1127,7 +1124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>1046</v>
       </c>
@@ -1141,7 +1138,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>1139</v>
       </c>
@@ -1155,7 +1152,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>1049</v>
       </c>
@@ -1169,7 +1166,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>1051</v>
       </c>
@@ -1183,7 +1180,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>1054</v>
       </c>
@@ -1197,7 +1194,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>1055</v>
       </c>
@@ -1211,7 +1208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>1056</v>
       </c>
@@ -1225,7 +1222,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>1061</v>
       </c>
@@ -1239,7 +1236,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>1062</v>
       </c>
@@ -1253,7 +1250,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>1063</v>
       </c>
@@ -1267,7 +1264,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>1068</v>
       </c>
@@ -1281,7 +1278,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>1069</v>
       </c>
@@ -1295,7 +1292,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>1070</v>
       </c>
@@ -1309,7 +1306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>1140</v>
       </c>
@@ -1323,7 +1320,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>1141</v>
       </c>
@@ -1337,7 +1334,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>1142</v>
       </c>
@@ -1351,7 +1348,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>1144</v>
       </c>
@@ -1365,7 +1362,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>1145</v>
       </c>
@@ -1379,7 +1376,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>1146</v>
       </c>
@@ -1393,7 +1390,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>1147</v>
       </c>
@@ -1407,7 +1404,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>1149</v>
       </c>
@@ -1421,7 +1418,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>1150</v>
       </c>
@@ -1435,7 +1432,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>1072</v>
       </c>
@@ -1449,7 +1446,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>1073</v>
       </c>
@@ -1463,7 +1460,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>1075</v>
       </c>
@@ -1477,7 +1474,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>1151</v>
       </c>
@@ -1491,7 +1488,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>1076</v>
       </c>
@@ -1505,7 +1502,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>1078</v>
       </c>
@@ -1519,7 +1516,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>1079</v>
       </c>
@@ -1533,7 +1530,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>1152</v>
       </c>
@@ -1547,7 +1544,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>1080</v>
       </c>
@@ -1561,7 +1558,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>1154</v>
       </c>
@@ -1575,7 +1572,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>1155</v>
       </c>
@@ -1589,7 +1586,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>1086</v>
       </c>
@@ -1603,7 +1600,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>1156</v>
       </c>
@@ -1617,7 +1614,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>1087</v>
       </c>
@@ -1631,7 +1628,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>1157</v>
       </c>
@@ -1645,7 +1642,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>1089</v>
       </c>
@@ -1659,7 +1656,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>1158</v>
       </c>
@@ -1673,7 +1670,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>1159</v>
       </c>
@@ -1687,7 +1684,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>1160</v>
       </c>
@@ -1701,7 +1698,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>1161</v>
       </c>
@@ -1715,7 +1712,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>1162</v>
       </c>
@@ -1729,7 +1726,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>1090</v>
       </c>
@@ -1743,7 +1740,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>1163</v>
       </c>
@@ -1757,7 +1754,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>1092</v>
       </c>
@@ -1771,7 +1768,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>1093</v>
       </c>
@@ -1785,7 +1782,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>1098</v>
       </c>
@@ -1799,7 +1796,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>1099</v>
       </c>
@@ -1813,7 +1810,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>1164</v>
       </c>
@@ -1827,7 +1824,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>1104</v>
       </c>
@@ -1841,7 +1838,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>1109</v>
       </c>
@@ -1855,7 +1852,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>1165</v>
       </c>
@@ -1869,7 +1866,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>1113</v>
       </c>
@@ -1883,7 +1880,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>1114</v>
       </c>
@@ -1897,7 +1894,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>1166</v>
       </c>
@@ -1911,7 +1908,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>1119</v>
       </c>
@@ -1925,7 +1922,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>1167</v>
       </c>
@@ -1939,7 +1936,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>1168</v>
       </c>
@@ -1953,7 +1950,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>1121</v>
       </c>
@@ -1967,7 +1964,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>1122</v>
       </c>
@@ -1981,7 +1978,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>1170</v>
       </c>
@@ -1995,7 +1992,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>1123</v>
       </c>
@@ -2009,7 +2006,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>1125</v>
       </c>
@@ -2023,7 +2020,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>1171</v>
       </c>
@@ -2037,7 +2034,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>1173</v>
       </c>
@@ -2051,7 +2048,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
         <v>1174</v>
       </c>

</xml_diff>